<commit_message>
Adaptive: Business Sponsor -> u_business_owner, start date from StartDate (Project Assigned only as fallback)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018Ctr8mgkRhw8W6DYxzjejb
</commit_message>
<xml_diff>
--- a/docs/rm_story_revised.xlsx
+++ b/docs/rm_story_revised.xlsx
@@ -658,10 +658,12 @@
 Shared Adaptive rules (set in STRY0067506, used by every Adaptive story): correlation_id = "ADAPTIVE:" + the record's API id (e.g. ADAPTIVE:/Project/abc123); parent_correlation_id is built the same way from the parent's id; staging columns arrive as u_&lt;name&gt;; all value conversion happens in the transform map.
 This story is complete when:
 - A Transform Map routes u_imp_adaptive_project to pm_project. Coalesce on correlation_id only.
-- Core fields map 1:1: Name, Project Manager, Start/End dates, Percent Complete.
-- User references (Project Manager, Business Owner, Executive Sponsor) match sys_user on email. Choice action = Ignore (never create users).
+- Core fields map 1:1: Name, Project Manager, Percent Complete. Planned Finish -&gt; end_date.
+- start_date = Adaptive StartDate (system field; the Data Source adds it to the CZQL SELECT). If blank, use Project Assigned and log it. Project Assigned is not mapped as the start date otherwise.
+- Business Sponsor (free text, may list several names) -&gt; u_business_owner: if it holds one name, match it to sys_user; if it holds several names or there is no match, leave the field empty and add the full text to work_notes. u_executive_sponsor is not mapped (Adaptive has no executive sponsor field).
+- Project Manager matches sys_user on email. Choice action = Ignore (never create users).
 - State and Phase: Choice action = Reject. A field map script converts Adaptive values using the value table below.
-- Custom fields u_business_owner, u_executive_sponsor, u_cn, u_sites, u_funding_type, u_funding_source, u_business_category map exactly as in the Demand map (STRY0066695).
+- Custom fields u_cn, u_sites, u_funding_type, u_funding_source, u_business_category map exactly as in the Demand map (STRY0066695).
 - u_sites: a field map script splits the site names and returns sys_ids from [BA TO CONFIRM - Sites table, see D3]. Unknown names are logged.
 - Running the same data a second time in sub-production inserts 0 new records.
 Adaptive State | ServiceNow state
@@ -673,7 +675,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Conversion now in the transform map (no upstream pipeline). Added u_executive_sponsor to match the Demand map. Added u_sites script and state value table.</t>
+          <t>Conversion now in the transform map (no upstream pipeline). Business Sponsor -&gt; u_business_owner; u_executive_sponsor left empty (no Adaptive source). Start date from Adaptive StartDate, not Project Assigned. Added u_sites script and state value table.</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
@@ -702,7 +704,7 @@
           <t>&lt;p&gt;Reference the &amp;quot;Project Mapping&amp;quot; tab in the attached Adaptive_to_ServiceNow_Mapping_Guide.xlsx for field-level directives. &amp;quot;Project fields for data migration.xlsx&amp;quot; shows an example Adaptive project.&lt;/p&gt;
 &lt;p&gt;Shared Adaptive rules (set in STRY0067506, used by every Adaptive story): correlation_id = &amp;quot;ADAPTIVE:&amp;quot; + the record&amp;#x27;s API id (e.g. ADAPTIVE:/Project/abc123); parent_correlation_id is built the same way from the parent&amp;#x27;s id; staging columns arrive as u_&amp;lt;name&amp;gt;; all value conversion happens in the transform map.&lt;/p&gt;
 &lt;p&gt;This story is complete when:&lt;/p&gt;
-&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;A Transform Map routes u_imp_adaptive_project to pm_project. Coalesce on correlation_id only.&lt;/li&gt;&lt;li&gt;Core fields map 1:1: Name, Project Manager, Start/End dates, Percent Complete.&lt;/li&gt;&lt;li&gt;User references (Project Manager, Business Owner, Executive Sponsor) match sys_user on email. Choice action = Ignore (never create users).&lt;/li&gt;&lt;li&gt;State and Phase: Choice action = Reject. A field map script converts Adaptive values using the value table below.&lt;/li&gt;&lt;li&gt;Custom fields u_business_owner, u_executive_sponsor, u_cn, u_sites, u_funding_type, u_funding_source, u_business_category map exactly as in the Demand map (STRY0066695).&lt;/li&gt;&lt;li&gt;u_sites: a field map script splits the site names and returns sys_ids from [BA TO CONFIRM - Sites table, see D3]. Unknown names are logged.&lt;/li&gt;&lt;li&gt;Running the same data a second time in sub-production inserts 0 new records.&lt;/li&gt;&lt;/ul&gt;
+&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;A Transform Map routes u_imp_adaptive_project to pm_project. Coalesce on correlation_id only.&lt;/li&gt;&lt;li&gt;Core fields map 1:1: Name, Project Manager, Percent Complete. Planned Finish -&amp;gt; end_date.&lt;/li&gt;&lt;li&gt;start_date = Adaptive StartDate (system field; the Data Source adds it to the CZQL SELECT). If blank, use Project Assigned and log it. Project Assigned is not mapped as the start date otherwise.&lt;/li&gt;&lt;li&gt;Business Sponsor (free text, may list several names) -&amp;gt; u_business_owner: if it holds one name, match it to sys_user; if it holds several names or there is no match, leave the field empty and add the full text to work_notes. u_executive_sponsor is not mapped (Adaptive has no executive sponsor field).&lt;/li&gt;&lt;li&gt;Project Manager matches sys_user on email. Choice action = Ignore (never create users).&lt;/li&gt;&lt;li&gt;State and Phase: Choice action = Reject. A field map script converts Adaptive values using the value table below.&lt;/li&gt;&lt;li&gt;Custom fields u_cn, u_sites, u_funding_type, u_funding_source, u_business_category map exactly as in the Demand map (STRY0066695).&lt;/li&gt;&lt;li&gt;u_sites: a field map script splits the site names and returns sys_ids from [BA TO CONFIRM - Sites table, see D3]. Unknown names are logged.&lt;/li&gt;&lt;li&gt;Running the same data a second time in sub-production inserts 0 new records.&lt;/li&gt;&lt;/ul&gt;
 &lt;table style="width: 100%;"&gt;&lt;thead&gt;&lt;tr&gt;&lt;td&gt;&lt;strong&gt;Adaptive State&lt;/strong&gt;&lt;/td&gt;&lt;td&gt;&lt;strong&gt;ServiceNow state&lt;/strong&gt;&lt;/td&gt;&lt;/tr&gt;&lt;/thead&gt;&lt;tbody&gt;&lt;tr&gt;&lt;td&gt;Draft&lt;/td&gt;&lt;td&gt;[BA TO CONFIRM - see D4]&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Requested&lt;/td&gt;&lt;td&gt;[BA TO CONFIRM - see D4]&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;Active&lt;/td&gt;&lt;td&gt;[BA TO CONFIRM - see D4]&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;On Hold&lt;/td&gt;&lt;td&gt;[BA TO CONFIRM - see D4]&lt;/td&gt;&lt;/tr&gt;&lt;/tbody&gt;&lt;/table&gt;</t>
         </is>
       </c>
@@ -795,9 +797,9 @@
 Blocked until the Demand vs Project rule is confirmed (D2).
 This story is complete when:
 - A Transform Map routes u_imp_adaptive_demand to dmn_demand. Coalesce on correlation_id only.
-- Name, Phase/State and Dates map 1:1. Choice action = Reject; a field map script converts Adaptive values to ServiceNow choices.
+- Name, Phase/State and Dates map 1:1 (start date and Business Sponsor follow the Project map rules). Choice action = Reject; a field map script converts Adaptive values to ServiceNow choices.
 - Capex Budget, Opex Budget and Total Budget map to the demand's matching budget fields (dev confirms the field names in the dictionary). Skip this if cost plans are loaded for demands [BA TO CONFIRM - see D5].
-- Custom fields u_business_owner, u_executive_sponsor, u_cn, u_funding_type, u_funding_source, u_business_category map 1:1.
+- Custom fields u_business_owner (from Business Sponsor), u_cn, u_funding_type, u_funding_source, u_business_category map 1:1.
 - u_sites uses the same field map script as the Project map (STRY0066697).
 - User references resolve on email (e.g. BusinessOwner.Email). Choice action = Ignore.
 - Running the same data a second time inserts 0 new records.</t>
@@ -835,7 +837,7 @@
 &lt;p&gt;Shared Adaptive rules (set in STRY0067506, used by every Adaptive story): correlation_id = &amp;quot;ADAPTIVE:&amp;quot; + the record&amp;#x27;s API id (e.g. ADAPTIVE:/Project/abc123); parent_correlation_id is built the same way from the parent&amp;#x27;s id; staging columns arrive as u_&amp;lt;name&amp;gt;; all value conversion happens in the transform map.&lt;/p&gt;
 &lt;p&gt;Blocked until the Demand vs Project rule is confirmed (D2).&lt;/p&gt;
 &lt;p&gt;This story is complete when:&lt;/p&gt;
-&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;A Transform Map routes u_imp_adaptive_demand to dmn_demand. Coalesce on correlation_id only.&lt;/li&gt;&lt;li&gt;Name, Phase/State and Dates map 1:1. Choice action = Reject; a field map script converts Adaptive values to ServiceNow choices.&lt;/li&gt;&lt;li&gt;Capex Budget, Opex Budget and Total Budget map to the demand&amp;#x27;s matching budget fields (dev confirms the field names in the dictionary). Skip this if cost plans are loaded for demands [BA TO CONFIRM - see D5].&lt;/li&gt;&lt;li&gt;Custom fields u_business_owner, u_executive_sponsor, u_cn, u_funding_type, u_funding_source, u_business_category map 1:1.&lt;/li&gt;&lt;li&gt;u_sites uses the same field map script as the Project map (STRY0066697).&lt;/li&gt;&lt;li&gt;User references resolve on email (e.g. BusinessOwner.Email). Choice action = Ignore.&lt;/li&gt;&lt;li&gt;Running the same data a second time inserts 0 new records.&lt;/li&gt;&lt;/ul&gt;</t>
+&lt;ul style="list-style-position: inside;"&gt;&lt;li&gt;A Transform Map routes u_imp_adaptive_demand to dmn_demand. Coalesce on correlation_id only.&lt;/li&gt;&lt;li&gt;Name, Phase/State and Dates map 1:1 (start date and Business Sponsor follow the Project map rules). Choice action = Reject; a field map script converts Adaptive values to ServiceNow choices.&lt;/li&gt;&lt;li&gt;Capex Budget, Opex Budget and Total Budget map to the demand&amp;#x27;s matching budget fields (dev confirms the field names in the dictionary). Skip this if cost plans are loaded for demands [BA TO CONFIRM - see D5].&lt;/li&gt;&lt;li&gt;Custom fields u_business_owner (from Business Sponsor), u_cn, u_funding_type, u_funding_source, u_business_category map 1:1.&lt;/li&gt;&lt;li&gt;u_sites uses the same field map script as the Project map (STRY0066697).&lt;/li&gt;&lt;li&gt;User references resolve on email (e.g. BusinessOwner.Email). Choice action = Ignore.&lt;/li&gt;&lt;li&gt;Running the same data a second time inserts 0 new records.&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>